<commit_message>
docs: certify combat data and party cycles
</commit_message>
<xml_diff>
--- a/docs/design/2026-09-04-project-design-tables/GameXXK_怪物与阶段数值设计总表_2026-09-04.xlsx
+++ b/docs/design/2026-09-04-project-design-tables/GameXXK_怪物与阶段数值设计总表_2026-09-04.xlsx
@@ -17,7 +17,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_阶段二意图" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_阶段三意图" sheetId="9" state="visible" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_数值换算" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_实现差异" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_实现状态" sheetId="11" state="visible" r:id="rId11"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_来源校验" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames>
@@ -31,7 +31,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'07_阶段二意图'!$A$1:$E$40</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'08_阶段三意图'!$A$1:$E$40</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'09_数值换算'!$A$1:$E$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'10_实现差异'!$A$1:$C$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'10_实现状态'!$A$1:$C$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'11_来源校验'!$A$1:$B$3</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -490,7 +490,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-03批准重平衡规格；旧EnemyCatalog意图/阶段与训练池冲突时以规格为准</t>
+          <t>2026-09-03批准重平衡规格；运行时目录、历练编制与本表按同一口径验证</t>
         </is>
       </c>
     </row>
@@ -550,7 +550,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>当前代码仍是旧Boss二阶段和旧池；本表是批准设计，不是当前运行时导出</t>
+          <t>v36已实装；351个难度/阶段意图预演、189组固定编制、阶段切换与存档迁移均有自动化证据</t>
         </is>
       </c>
     </row>
@@ -781,7 +781,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="62" customWidth="1" min="2" max="2"/>
+    <col width="76" customWidth="1" min="2" max="2"/>
     <col width="90" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
@@ -793,12 +793,12 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>当前旧实现</t>
+          <t>当前实现</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>批准设计</t>
+          <t>验证口径</t>
         </is>
       </c>
     </row>
@@ -810,12 +810,12 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>使用玩家等级/旧路线夹具</t>
+          <t>固定5..135；战斗和游历均读取关卡CombatLevel</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>固定5..135关卡等级；地狱3-1=125</t>
+          <t>地狱3-1=125；地狱3-3=135</t>
         </is>
       </c>
     </row>
@@ -827,12 +827,12 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>未完整进入卡牌战斗</t>
+          <t>显式Normal/Hard/Hell并校验100/125/150%</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>普通/困难/地狱伤害100/125/150%</t>
+          <t>预演与执行读取同一枚举</t>
         </is>
       </c>
     </row>
@@ -844,12 +844,12 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Boss专用bPhaseTwo</t>
+          <t>九名精英/首领按难度使用1/2/3阶段</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>九名精英/首领数据驱动1/2/3阶段</t>
+          <t>阶段牌组连续且旧Intents为空</t>
         </is>
       </c>
     </row>
@@ -861,12 +861,12 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>半血标记并可能改属性</t>
+          <t>伤害包截断至1HP、满血新阶段、清负面、保正面与护甲</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>伤害包安全截断、满血新阶段、清负面、保正面、换整套牌</t>
+          <t>直伤、多段、DOT、反击共用规则</t>
         </is>
       </c>
     </row>
@@ -878,12 +878,12 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>平行池临时组合</t>
+          <t>27关×7=189组固定左中右与开场意图</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>27关×7=189组固定左中右与开场意图</t>
+          <t>挑战与游历读取同一EnemySlots</t>
         </is>
       </c>
     </row>
@@ -895,12 +895,12 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>旧目录78意图</t>
+          <t>36普通、42阶段一、39阶段二、39阶段三</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>351个难度/阶段解析用例</t>
+          <t>108+126+78+39=351预演通过</t>
         </is>
       </c>
     </row>
@@ -912,12 +912,12 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>旧第三章路线普通/精英/Boss夹具</t>
+          <t>125级 秃鹫-白猿-巨蟾，阶段1/3/1</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>125级 秃鹫-白猿-巨蟾，阶段1/3/1，总阶段生命11178</t>
+          <t>总原始阶段生命11178</t>
         </is>
       </c>
     </row>
@@ -972,7 +972,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>e3db4e38ec589b68e41c2e15e45bd44f5853d0d048a0b4084078a44d7e06f47c</t>
+          <t>b3bdee311b086dd6d2e33bf95125d8173de04696345a45c5f4ecb8f9a3fe69d2</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: back up shared GameXXK work (1/21)
</commit_message>
<xml_diff>
--- a/docs/design/2026-09-04-project-design-tables/GameXXK_怪物与阶段数值设计总表_2026-09-04.xlsx
+++ b/docs/design/2026-09-04-project-design-tables/GameXXK_怪物与阶段数值设计总表_2026-09-04.xlsx
@@ -19,6 +19,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_数值换算" sheetId="10" state="visible" r:id="rId10"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_实现状态" sheetId="11" state="visible" r:id="rId11"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_来源校验" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14_挂机金币曲线" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'00_说明'!$A$1:$B$7</definedName>
@@ -33,6 +34,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'09_数值换算'!$A$1:$E$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'10_实现状态'!$A$1:$C$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'11_来源校验'!$A$1:$B$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'14_挂机金币曲线'!$A$1:$H$28</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -41,7 +43,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -59,8 +61,19 @@
       <name val="微软雅黑"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Microsoft YaHei"/>
+      <color rgb="00263F43"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Microsoft YaHei"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -70,6 +83,21 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001F4E78"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F1F5F4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00244D57"/>
       </patternFill>
     </fill>
   </fills>
@@ -90,13 +118,28 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -982,6 +1025,991 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H28"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="21" customWidth="1" min="4" max="4"/>
+    <col width="21" customWidth="1" min="5" max="5"/>
+    <col width="31" customWidth="1" min="6" max="6"/>
+    <col width="70" customWidth="1" min="7" max="7"/>
+    <col width="68" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>难度</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>关卡</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>敌人等级</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>每波基础金币</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>每波基础经验</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>满在线金币天赋每波金币</t>
+        </is>
+      </c>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>当前状态</t>
+        </is>
+      </c>
+      <c r="H1" s="3" t="inlineStr">
+        <is>
+          <t>源码定位</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="38" customHeight="1">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>普通</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="D2" s="5" t="n">
+        <v>210</v>
+      </c>
+      <c r="E2" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="F2" s="5" t="n">
+        <v>945</v>
+      </c>
+      <c r="G2" s="4" t="inlineStr">
+        <is>
+          <t>已校准：普通×10；困难至地狱连续每关×1.05；天赋价格与45天基准见07E/07F</t>
+        </is>
+      </c>
+      <c r="H2" s="4" t="inlineStr">
+        <is>
+          <t>Source/GameXXK/Private/GameXXKTrainingRules.cpp；docs/design/2026-09-10-training-gold-talent-calibration.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="38" customHeight="1">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>普通</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="D3" s="7" t="n">
+        <v>240</v>
+      </c>
+      <c r="E3" s="7" t="n">
+        <v>14</v>
+      </c>
+      <c r="F3" s="7" t="n">
+        <v>1080</v>
+      </c>
+      <c r="G3" s="6" t="inlineStr">
+        <is>
+          <t>已校准：普通×10；困难至地狱连续每关×1.05；天赋价格与45天基准见07E/07F</t>
+        </is>
+      </c>
+      <c r="H3" s="6" t="inlineStr">
+        <is>
+          <t>Source/GameXXK/Private/GameXXKTrainingRules.cpp；docs/design/2026-09-10-training-gold-talent-calibration.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="38" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>普通</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>1-3</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="D4" s="5" t="n">
+        <v>270</v>
+      </c>
+      <c r="E4" s="5" t="n">
+        <v>16</v>
+      </c>
+      <c r="F4" s="5" t="n">
+        <v>1215</v>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>已校准：普通×10；困难至地狱连续每关×1.05；天赋价格与45天基准见07E/07F</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>Source/GameXXK/Private/GameXXKTrainingRules.cpp；docs/design/2026-09-10-training-gold-talent-calibration.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="38" customHeight="1">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>普通</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="n">
+        <v>20</v>
+      </c>
+      <c r="D5" s="7" t="n">
+        <v>300</v>
+      </c>
+      <c r="E5" s="7" t="n">
+        <v>18</v>
+      </c>
+      <c r="F5" s="7" t="n">
+        <v>1350</v>
+      </c>
+      <c r="G5" s="6" t="inlineStr">
+        <is>
+          <t>已校准：普通×10；困难至地狱连续每关×1.05；天赋价格与45天基准见07E/07F</t>
+        </is>
+      </c>
+      <c r="H5" s="6" t="inlineStr">
+        <is>
+          <t>Source/GameXXK/Private/GameXXKTrainingRules.cpp；docs/design/2026-09-10-training-gold-talent-calibration.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="38" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>普通</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>2-2</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="D6" s="5" t="n">
+        <v>330</v>
+      </c>
+      <c r="E6" s="5" t="n">
+        <v>20</v>
+      </c>
+      <c r="F6" s="5" t="n">
+        <v>1485</v>
+      </c>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>已校准：普通×10；困难至地狱连续每关×1.05；天赋价格与45天基准见07E/07F</t>
+        </is>
+      </c>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>Source/GameXXK/Private/GameXXKTrainingRules.cpp；docs/design/2026-09-10-training-gold-talent-calibration.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="38" customHeight="1">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>普通</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>2-3</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="n">
+        <v>30</v>
+      </c>
+      <c r="D7" s="7" t="n">
+        <v>360</v>
+      </c>
+      <c r="E7" s="7" t="n">
+        <v>22</v>
+      </c>
+      <c r="F7" s="7" t="n">
+        <v>1620</v>
+      </c>
+      <c r="G7" s="6" t="inlineStr">
+        <is>
+          <t>已校准：普通×10；困难至地狱连续每关×1.05；天赋价格与45天基准见07E/07F</t>
+        </is>
+      </c>
+      <c r="H7" s="6" t="inlineStr">
+        <is>
+          <t>Source/GameXXK/Private/GameXXKTrainingRules.cpp；docs/design/2026-09-10-training-gold-talent-calibration.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="38" customHeight="1">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>普通</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>3-1</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="n">
+        <v>35</v>
+      </c>
+      <c r="D8" s="5" t="n">
+        <v>390</v>
+      </c>
+      <c r="E8" s="5" t="n">
+        <v>24</v>
+      </c>
+      <c r="F8" s="5" t="n">
+        <v>1755</v>
+      </c>
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>已校准：普通×10；困难至地狱连续每关×1.05；天赋价格与45天基准见07E/07F</t>
+        </is>
+      </c>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>Source/GameXXK/Private/GameXXKTrainingRules.cpp；docs/design/2026-09-10-training-gold-talent-calibration.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="38" customHeight="1">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>普通</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>3-2</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="n">
+        <v>40</v>
+      </c>
+      <c r="D9" s="7" t="n">
+        <v>420</v>
+      </c>
+      <c r="E9" s="7" t="n">
+        <v>26</v>
+      </c>
+      <c r="F9" s="7" t="n">
+        <v>1890</v>
+      </c>
+      <c r="G9" s="6" t="inlineStr">
+        <is>
+          <t>已校准：普通×10；困难至地狱连续每关×1.05；天赋价格与45天基准见07E/07F</t>
+        </is>
+      </c>
+      <c r="H9" s="6" t="inlineStr">
+        <is>
+          <t>Source/GameXXK/Private/GameXXKTrainingRules.cpp；docs/design/2026-09-10-training-gold-talent-calibration.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="38" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>普通</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>3-3</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="D10" s="5" t="n">
+        <v>450</v>
+      </c>
+      <c r="E10" s="5" t="n">
+        <v>28</v>
+      </c>
+      <c r="F10" s="5" t="n">
+        <v>2025</v>
+      </c>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>已校准：普通×10；困难至地狱连续每关×1.05；天赋价格与45天基准见07E/07F</t>
+        </is>
+      </c>
+      <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t>Source/GameXXK/Private/GameXXKTrainingRules.cpp；docs/design/2026-09-10-training-gold-talent-calibration.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="38" customHeight="1">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>困难</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="n">
+        <v>50</v>
+      </c>
+      <c r="D11" s="7" t="n">
+        <v>473</v>
+      </c>
+      <c r="E11" s="7" t="n">
+        <v>22</v>
+      </c>
+      <c r="F11" s="7" t="n">
+        <v>2129</v>
+      </c>
+      <c r="G11" s="6" t="inlineStr">
+        <is>
+          <t>已校准：普通×10；困难至地狱连续每关×1.05；天赋价格与45天基准见07E/07F</t>
+        </is>
+      </c>
+      <c r="H11" s="6" t="inlineStr">
+        <is>
+          <t>Source/GameXXK/Private/GameXXKTrainingRules.cpp；docs/design/2026-09-10-training-gold-talent-calibration.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="38" customHeight="1">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>困难</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="n">
+        <v>55</v>
+      </c>
+      <c r="D12" s="5" t="n">
+        <v>496</v>
+      </c>
+      <c r="E12" s="5" t="n">
+        <v>24</v>
+      </c>
+      <c r="F12" s="5" t="n">
+        <v>2232</v>
+      </c>
+      <c r="G12" s="4" t="inlineStr">
+        <is>
+          <t>已校准：普通×10；困难至地狱连续每关×1.05；天赋价格与45天基准见07E/07F</t>
+        </is>
+      </c>
+      <c r="H12" s="4" t="inlineStr">
+        <is>
+          <t>Source/GameXXK/Private/GameXXKTrainingRules.cpp；docs/design/2026-09-10-training-gold-talent-calibration.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="38" customHeight="1">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>困难</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>1-3</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="n">
+        <v>60</v>
+      </c>
+      <c r="D13" s="7" t="n">
+        <v>521</v>
+      </c>
+      <c r="E13" s="7" t="n">
+        <v>26</v>
+      </c>
+      <c r="F13" s="7" t="n">
+        <v>2345</v>
+      </c>
+      <c r="G13" s="6" t="inlineStr">
+        <is>
+          <t>已校准：普通×10；困难至地狱连续每关×1.05；天赋价格与45天基准见07E/07F</t>
+        </is>
+      </c>
+      <c r="H13" s="6" t="inlineStr">
+        <is>
+          <t>Source/GameXXK/Private/GameXXKTrainingRules.cpp；docs/design/2026-09-10-training-gold-talent-calibration.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="38" customHeight="1">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>困难</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="n">
+        <v>65</v>
+      </c>
+      <c r="D14" s="5" t="n">
+        <v>547</v>
+      </c>
+      <c r="E14" s="5" t="n">
+        <v>28</v>
+      </c>
+      <c r="F14" s="5" t="n">
+        <v>2462</v>
+      </c>
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>已校准：普通×10；困难至地狱连续每关×1.05；天赋价格与45天基准见07E/07F</t>
+        </is>
+      </c>
+      <c r="H14" s="4" t="inlineStr">
+        <is>
+          <t>Source/GameXXK/Private/GameXXKTrainingRules.cpp；docs/design/2026-09-10-training-gold-talent-calibration.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="38" customHeight="1">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>困难</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>2-2</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="n">
+        <v>70</v>
+      </c>
+      <c r="D15" s="7" t="n">
+        <v>574</v>
+      </c>
+      <c r="E15" s="7" t="n">
+        <v>30</v>
+      </c>
+      <c r="F15" s="7" t="n">
+        <v>2583</v>
+      </c>
+      <c r="G15" s="6" t="inlineStr">
+        <is>
+          <t>已校准：普通×10；困难至地狱连续每关×1.05；天赋价格与45天基准见07E/07F</t>
+        </is>
+      </c>
+      <c r="H15" s="6" t="inlineStr">
+        <is>
+          <t>Source/GameXXK/Private/GameXXKTrainingRules.cpp；docs/design/2026-09-10-training-gold-talent-calibration.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="38" customHeight="1">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>困难</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>2-3</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="n">
+        <v>75</v>
+      </c>
+      <c r="D16" s="5" t="n">
+        <v>603</v>
+      </c>
+      <c r="E16" s="5" t="n">
+        <v>32</v>
+      </c>
+      <c r="F16" s="5" t="n">
+        <v>2714</v>
+      </c>
+      <c r="G16" s="4" t="inlineStr">
+        <is>
+          <t>已校准：普通×10；困难至地狱连续每关×1.05；天赋价格与45天基准见07E/07F</t>
+        </is>
+      </c>
+      <c r="H16" s="4" t="inlineStr">
+        <is>
+          <t>Source/GameXXK/Private/GameXXKTrainingRules.cpp；docs/design/2026-09-10-training-gold-talent-calibration.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="38" customHeight="1">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>困难</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>3-1</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="n">
+        <v>80</v>
+      </c>
+      <c r="D17" s="7" t="n">
+        <v>633</v>
+      </c>
+      <c r="E17" s="7" t="n">
+        <v>34</v>
+      </c>
+      <c r="F17" s="7" t="n">
+        <v>2849</v>
+      </c>
+      <c r="G17" s="6" t="inlineStr">
+        <is>
+          <t>已校准：普通×10；困难至地狱连续每关×1.05；天赋价格与45天基准见07E/07F</t>
+        </is>
+      </c>
+      <c r="H17" s="6" t="inlineStr">
+        <is>
+          <t>Source/GameXXK/Private/GameXXKTrainingRules.cpp；docs/design/2026-09-10-training-gold-talent-calibration.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="38" customHeight="1">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>困难</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>3-2</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="n">
+        <v>85</v>
+      </c>
+      <c r="D18" s="5" t="n">
+        <v>665</v>
+      </c>
+      <c r="E18" s="5" t="n">
+        <v>36</v>
+      </c>
+      <c r="F18" s="5" t="n">
+        <v>2993</v>
+      </c>
+      <c r="G18" s="4" t="inlineStr">
+        <is>
+          <t>已校准：普通×10；困难至地狱连续每关×1.05；天赋价格与45天基准见07E/07F</t>
+        </is>
+      </c>
+      <c r="H18" s="4" t="inlineStr">
+        <is>
+          <t>Source/GameXXK/Private/GameXXKTrainingRules.cpp；docs/design/2026-09-10-training-gold-talent-calibration.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="38" customHeight="1">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>困难</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>3-3</t>
+        </is>
+      </c>
+      <c r="C19" s="7" t="n">
+        <v>90</v>
+      </c>
+      <c r="D19" s="7" t="n">
+        <v>698</v>
+      </c>
+      <c r="E19" s="7" t="n">
+        <v>38</v>
+      </c>
+      <c r="F19" s="7" t="n">
+        <v>3141</v>
+      </c>
+      <c r="G19" s="6" t="inlineStr">
+        <is>
+          <t>已校准：普通×10；困难至地狱连续每关×1.05；天赋价格与45天基准见07E/07F</t>
+        </is>
+      </c>
+      <c r="H19" s="6" t="inlineStr">
+        <is>
+          <t>Source/GameXXK/Private/GameXXKTrainingRules.cpp；docs/design/2026-09-10-training-gold-talent-calibration.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="38" customHeight="1">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>地狱</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="n">
+        <v>95</v>
+      </c>
+      <c r="D20" s="5" t="n">
+        <v>733</v>
+      </c>
+      <c r="E20" s="5" t="n">
+        <v>32</v>
+      </c>
+      <c r="F20" s="5" t="n">
+        <v>3299</v>
+      </c>
+      <c r="G20" s="4" t="inlineStr">
+        <is>
+          <t>已校准：普通×10；困难至地狱连续每关×1.05；天赋价格与45天基准见07E/07F</t>
+        </is>
+      </c>
+      <c r="H20" s="4" t="inlineStr">
+        <is>
+          <t>Source/GameXXK/Private/GameXXKTrainingRules.cpp；docs/design/2026-09-10-training-gold-talent-calibration.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="38" customHeight="1">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>地狱</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="n">
+        <v>100</v>
+      </c>
+      <c r="D21" s="7" t="n">
+        <v>770</v>
+      </c>
+      <c r="E21" s="7" t="n">
+        <v>34</v>
+      </c>
+      <c r="F21" s="7" t="n">
+        <v>3465</v>
+      </c>
+      <c r="G21" s="6" t="inlineStr">
+        <is>
+          <t>已校准：普通×10；困难至地狱连续每关×1.05；天赋价格与45天基准见07E/07F</t>
+        </is>
+      </c>
+      <c r="H21" s="6" t="inlineStr">
+        <is>
+          <t>Source/GameXXK/Private/GameXXKTrainingRules.cpp；docs/design/2026-09-10-training-gold-talent-calibration.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="38" customHeight="1">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>地狱</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>1-3</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="n">
+        <v>105</v>
+      </c>
+      <c r="D22" s="5" t="n">
+        <v>808</v>
+      </c>
+      <c r="E22" s="5" t="n">
+        <v>36</v>
+      </c>
+      <c r="F22" s="5" t="n">
+        <v>3636</v>
+      </c>
+      <c r="G22" s="4" t="inlineStr">
+        <is>
+          <t>已校准：普通×10；困难至地狱连续每关×1.05；天赋价格与45天基准见07E/07F</t>
+        </is>
+      </c>
+      <c r="H22" s="4" t="inlineStr">
+        <is>
+          <t>Source/GameXXK/Private/GameXXKTrainingRules.cpp；docs/design/2026-09-10-training-gold-talent-calibration.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="38" customHeight="1">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t>地狱</t>
+        </is>
+      </c>
+      <c r="B23" s="6" t="inlineStr">
+        <is>
+          <t>2-1</t>
+        </is>
+      </c>
+      <c r="C23" s="7" t="n">
+        <v>110</v>
+      </c>
+      <c r="D23" s="7" t="n">
+        <v>849</v>
+      </c>
+      <c r="E23" s="7" t="n">
+        <v>38</v>
+      </c>
+      <c r="F23" s="7" t="n">
+        <v>3821</v>
+      </c>
+      <c r="G23" s="6" t="inlineStr">
+        <is>
+          <t>已校准：普通×10；困难至地狱连续每关×1.05；天赋价格与45天基准见07E/07F</t>
+        </is>
+      </c>
+      <c r="H23" s="6" t="inlineStr">
+        <is>
+          <t>Source/GameXXK/Private/GameXXKTrainingRules.cpp；docs/design/2026-09-10-training-gold-talent-calibration.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="38" customHeight="1">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>地狱</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>2-2</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="n">
+        <v>115</v>
+      </c>
+      <c r="D24" s="5" t="n">
+        <v>891</v>
+      </c>
+      <c r="E24" s="5" t="n">
+        <v>40</v>
+      </c>
+      <c r="F24" s="5" t="n">
+        <v>4010</v>
+      </c>
+      <c r="G24" s="4" t="inlineStr">
+        <is>
+          <t>已校准：普通×10；困难至地狱连续每关×1.05；天赋价格与45天基准见07E/07F</t>
+        </is>
+      </c>
+      <c r="H24" s="4" t="inlineStr">
+        <is>
+          <t>Source/GameXXK/Private/GameXXKTrainingRules.cpp；docs/design/2026-09-10-training-gold-talent-calibration.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="38" customHeight="1">
+      <c r="A25" s="6" t="inlineStr">
+        <is>
+          <t>地狱</t>
+        </is>
+      </c>
+      <c r="B25" s="6" t="inlineStr">
+        <is>
+          <t>2-3</t>
+        </is>
+      </c>
+      <c r="C25" s="7" t="n">
+        <v>120</v>
+      </c>
+      <c r="D25" s="7" t="n">
+        <v>936</v>
+      </c>
+      <c r="E25" s="7" t="n">
+        <v>42</v>
+      </c>
+      <c r="F25" s="7" t="n">
+        <v>4212</v>
+      </c>
+      <c r="G25" s="6" t="inlineStr">
+        <is>
+          <t>已校准：普通×10；困难至地狱连续每关×1.05；天赋价格与45天基准见07E/07F</t>
+        </is>
+      </c>
+      <c r="H25" s="6" t="inlineStr">
+        <is>
+          <t>Source/GameXXK/Private/GameXXKTrainingRules.cpp；docs/design/2026-09-10-training-gold-talent-calibration.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="38" customHeight="1">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>地狱</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>3-1</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="n">
+        <v>125</v>
+      </c>
+      <c r="D26" s="5" t="n">
+        <v>982</v>
+      </c>
+      <c r="E26" s="5" t="n">
+        <v>44</v>
+      </c>
+      <c r="F26" s="5" t="n">
+        <v>4419</v>
+      </c>
+      <c r="G26" s="4" t="inlineStr">
+        <is>
+          <t>已校准：普通×10；困难至地狱连续每关×1.05；天赋价格与45天基准见07E/07F</t>
+        </is>
+      </c>
+      <c r="H26" s="4" t="inlineStr">
+        <is>
+          <t>Source/GameXXK/Private/GameXXKTrainingRules.cpp；docs/design/2026-09-10-training-gold-talent-calibration.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="38" customHeight="1">
+      <c r="A27" s="6" t="inlineStr">
+        <is>
+          <t>地狱</t>
+        </is>
+      </c>
+      <c r="B27" s="6" t="inlineStr">
+        <is>
+          <t>3-2</t>
+        </is>
+      </c>
+      <c r="C27" s="7" t="n">
+        <v>130</v>
+      </c>
+      <c r="D27" s="7" t="n">
+        <v>1031</v>
+      </c>
+      <c r="E27" s="7" t="n">
+        <v>46</v>
+      </c>
+      <c r="F27" s="7" t="n">
+        <v>4640</v>
+      </c>
+      <c r="G27" s="6" t="inlineStr">
+        <is>
+          <t>已校准：普通×10；困难至地狱连续每关×1.05；天赋价格与45天基准见07E/07F</t>
+        </is>
+      </c>
+      <c r="H27" s="6" t="inlineStr">
+        <is>
+          <t>Source/GameXXK/Private/GameXXKTrainingRules.cpp；docs/design/2026-09-10-training-gold-talent-calibration.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="38" customHeight="1">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>地狱</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>3-3</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="n">
+        <v>135</v>
+      </c>
+      <c r="D28" s="5" t="n">
+        <v>1083</v>
+      </c>
+      <c r="E28" s="5" t="n">
+        <v>48</v>
+      </c>
+      <c r="F28" s="5" t="n">
+        <v>4874</v>
+      </c>
+      <c r="G28" s="4" t="inlineStr">
+        <is>
+          <t>已校准：普通×10；困难至地狱连续每关×1.05；天赋价格与45天基准见07E/07F</t>
+        </is>
+      </c>
+      <c r="H28" s="4" t="inlineStr">
+        <is>
+          <t>Source/GameXXK/Private/GameXXKTrainingRules.cpp；docs/design/2026-09-10-training-gold-talent-calibration.md</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:H28"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
chore: back up current gameplay, F10 tools, localization and art
</commit_message>
<xml_diff>
--- a/docs/design/2026-09-04-project-design-tables/GameXXK_怪物与阶段数值设计总表_2026-09-04.xlsx
+++ b/docs/design/2026-09-04-project-design-tables/GameXXK_怪物与阶段数值设计总表_2026-09-04.xlsx
@@ -23,7 +23,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'00_说明'!$A$1:$B$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'01_怪物属性'!$A$1:$T$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'01_怪物属性'!$A$1:$U$22</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'02_27关总表'!$A$1:$H$28</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'03_189编制'!$A$1:$I$190</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'04_地狱3-1'!$A$1:$G$8</definedName>
@@ -43,7 +43,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -72,8 +72,17 @@
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Microsoft YaHei"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <name val="Microsoft YaHei"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -100,6 +109,11 @@
         <fgColor rgb="00244D57"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00244C45"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -118,7 +132,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -139,6 +153,10 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="3" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2016,7 +2034,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T22"/>
+  <dimension ref="A1:U22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2039,6 +2057,7 @@
     <col width="10" customWidth="1" min="18" max="18"/>
     <col width="10" customWidth="1" min="19" max="19"/>
     <col width="10" customWidth="1" min="20" max="20"/>
+    <col width="28" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -2142,6 +2161,11 @@
           <t>L135防御</t>
         </is>
       </c>
+      <c r="U1" s="8" t="inlineStr">
+        <is>
+          <t>英文名称</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -2210,6 +2234,11 @@
       <c r="T2" s="2" t="n">
         <v>35</v>
       </c>
+      <c r="U2" s="9" t="inlineStr">
+        <is>
+          <t>Rooster</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -2278,6 +2307,11 @@
       <c r="T3" s="2" t="n">
         <v>50</v>
       </c>
+      <c r="U3" s="9" t="inlineStr">
+        <is>
+          <t>Goat</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -2346,6 +2380,11 @@
       <c r="T4" s="2" t="n">
         <v>28</v>
       </c>
+      <c r="U4" s="9" t="inlineStr">
+        <is>
+          <t>Weasel</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -2414,6 +2453,11 @@
       <c r="T5" s="2" t="n">
         <v>36</v>
       </c>
+      <c r="U5" s="9" t="inlineStr">
+        <is>
+          <t>Civet</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -2482,6 +2526,11 @@
       <c r="T6" s="2" t="n">
         <v>72</v>
       </c>
+      <c r="U6" s="9" t="inlineStr">
+        <is>
+          <t>Iron Rooster</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -2550,6 +2599,11 @@
       <c r="T7" s="2" t="n">
         <v>94</v>
       </c>
+      <c r="U7" s="9" t="inlineStr">
+        <is>
+          <t>Goat King</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -2618,6 +2672,11 @@
       <c r="T8" s="2" t="n">
         <v>109</v>
       </c>
+      <c r="U8" s="9" t="inlineStr">
+        <is>
+          <t>Money Rat</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -2686,6 +2745,11 @@
       <c r="T9" s="2" t="n">
         <v>42</v>
       </c>
+      <c r="U9" s="9" t="inlineStr">
+        <is>
+          <t>Gray Wolf</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -2754,6 +2818,11 @@
       <c r="T10" s="2" t="n">
         <v>65</v>
       </c>
+      <c r="U10" s="9" t="inlineStr">
+        <is>
+          <t>Boar</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -2822,6 +2891,11 @@
       <c r="T11" s="2" t="n">
         <v>36</v>
       </c>
+      <c r="U11" s="9" t="inlineStr">
+        <is>
+          <t>Macaque</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -2890,6 +2964,11 @@
       <c r="T12" s="2" t="n">
         <v>72</v>
       </c>
+      <c r="U12" s="9" t="inlineStr">
+        <is>
+          <t>Porcupine</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -2958,6 +3037,11 @@
       <c r="T13" s="2" t="n">
         <v>80</v>
       </c>
+      <c r="U13" s="9" t="inlineStr">
+        <is>
+          <t>Wolf King</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
@@ -3026,6 +3110,11 @@
       <c r="T14" s="2" t="n">
         <v>110</v>
       </c>
+      <c r="U14" s="9" t="inlineStr">
+        <is>
+          <t>Boar King</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
@@ -3094,6 +3183,11 @@
       <c r="T15" s="2" t="n">
         <v>132</v>
       </c>
+      <c r="U15" s="9" t="inlineStr">
+        <is>
+          <t>Black Bear</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
@@ -3162,6 +3256,11 @@
       <c r="T16" s="2" t="n">
         <v>36</v>
       </c>
+      <c r="U16" s="9" t="inlineStr">
+        <is>
+          <t>Venom Snake</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
@@ -3230,6 +3329,11 @@
       <c r="T17" s="2" t="n">
         <v>43</v>
       </c>
+      <c r="U17" s="9" t="inlineStr">
+        <is>
+          <t>Wildcat</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
@@ -3298,6 +3402,11 @@
       <c r="T18" s="2" t="n">
         <v>43</v>
       </c>
+      <c r="U18" s="9" t="inlineStr">
+        <is>
+          <t>Vulture</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
@@ -3366,6 +3475,11 @@
       <c r="T19" s="2" t="n">
         <v>87</v>
       </c>
+      <c r="U19" s="9" t="inlineStr">
+        <is>
+          <t>Giant Toad</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
@@ -3434,6 +3548,11 @@
       <c r="T20" s="2" t="n">
         <v>95</v>
       </c>
+      <c r="U20" s="9" t="inlineStr">
+        <is>
+          <t>White Ape</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
@@ -3502,6 +3621,11 @@
       <c r="T21" s="2" t="n">
         <v>110</v>
       </c>
+      <c r="U21" s="9" t="inlineStr">
+        <is>
+          <t>Spiral Deer</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
@@ -3570,9 +3694,14 @@
       <c r="T22" s="2" t="n">
         <v>146</v>
       </c>
+      <c r="U22" s="9" t="inlineStr">
+        <is>
+          <t>Tiger</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:T22"/>
+  <autoFilter ref="A1:U22"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
backup: preserve body-font rollout, source font and package reports
</commit_message>
<xml_diff>
--- a/docs/design/2026-09-04-project-design-tables/GameXXK_怪物与阶段数值设计总表_2026-09-04.xlsx
+++ b/docs/design/2026-09-04-project-design-tables/GameXXK_怪物与阶段数值设计总表_2026-09-04.xlsx
@@ -1,25 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_说明" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_怪物属性" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_27关总表" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_189编制" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_地狱3-1" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_普通怪意图" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_阶段一意图" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_阶段二意图" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_阶段三意图" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_数值换算" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_实现状态" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_来源校验" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14_挂机金币曲线" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="00_说明" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="01_怪物属性" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="02_27关总表" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="03_189编制" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="04_地狱3-1" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="05_普通怪意图" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="06_阶段一意图" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="07_阶段二意图" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="08_阶段三意图" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="09_数值换算" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="10_实现状态" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="11_来源校验" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="14_挂机金币曲线" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'00_说明'!$A$1:$B$7</definedName>

</xml_diff>